<commit_message>
updated publications 2025 to 2026
</commit_message>
<xml_diff>
--- a/publications.xlsx
+++ b/publications.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/g.s.collins@bham.ac.uk/git/personal-website/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/g.s.collins@bham.ac.uk/git/personal_pages/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E90211BF-9D05-0F4D-B9BB-529FF2E5B425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02F7D099-E7BE-964C-A2C6-8A642D6E4059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="45600" yWindow="600" windowWidth="22060" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="46580" yWindow="600" windowWidth="22060" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Publications" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="470">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="525">
   <si>
     <t>Section</t>
   </si>
@@ -1430,15 +1430,262 @@
   </si>
   <si>
     <t>2025, prediction models, sample size, meta-science</t>
+  </si>
+  <si>
+    <t>2025-04-15</t>
+  </si>
+  <si>
+    <t>CONSORT 2025 statement: updated guideline for reporting randomised trials</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1136/bmj-2024-081123</t>
+  </si>
+  <si>
+    <t>e081123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1136/bmj-2024-081123 </t>
+  </si>
+  <si>
+    <t>https://www.bmj.com/content/389/bmj-2024-081123.full.pdf</t>
+  </si>
+  <si>
+    <t>10.1001/jama.2025.4347</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1001/jama.2025.4347</t>
+  </si>
+  <si>
+    <t>1998-2005</t>
+  </si>
+  <si>
+    <t>10.1038/s41591-025-03635-5</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1038/s41591-025-03635-5</t>
+  </si>
+  <si>
+    <t>1776-1783</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41591-025-03635-5.pdf</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1371/journal.pmed.1004587</t>
+  </si>
+  <si>
+    <t>PLoS Medicine</t>
+  </si>
+  <si>
+    <t>e1004587</t>
+  </si>
+  <si>
+    <t>10.1371/journal.pmed.1004587</t>
+  </si>
+  <si>
+    <t>https://journals.plos.org/plosmedicine/article/file?id=10.1371/journal.pmed.1004587&amp;type=printable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONSORT 2025 Explanation and Elaboration: updated guideline for reporting randomised trials. </t>
+  </si>
+  <si>
+    <t>https://www.bmj.com/content/389/bmj-2024-081124.full.pdf</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1136/bmj-2024-081124</t>
+  </si>
+  <si>
+    <t>e081124</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1136/bmj-2024-081124 </t>
+  </si>
+  <si>
+    <r>
+      <t>Chan AW, Boutron I, Hopewell S,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Moher D,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Schulz KF, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>**Collins GS**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Tunn R, Aggarwal R, Berlin JA, Bhandari N, Butcher NJ, Campbell MK, Chidebe R, Elbourne D, Farmer A, Fergusson D, Golub RM, Goodman SN, Hoffmann T, Ioannidis JPA, Kahan B, Knowles R, Lamb SE, Lewis S, Loder E, Offringa M, Ravaud P, Richards D, Rockhold FW, Schriger DL, Siegfried N, Staniszewska S, Taylor R, Thabane L, Torgerson D, Vohra S, White IR, Hróbjartsson A.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>SPIRIT 2025 Statement: updated guideline for protocols of randomised trials</t>
+  </si>
+  <si>
+    <t>10.1136/bmj-2024-081477</t>
+  </si>
+  <si>
+    <t>https://www.bmj.com/content/389/bmj-2024-081477.full.pdf</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1136/bmj-2024-081477</t>
+  </si>
+  <si>
+    <t>2025, reporting guideline, CONSORT, trials, protocols</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1001/jama.2025.4486</t>
+  </si>
+  <si>
+    <t>435-443</t>
+  </si>
+  <si>
+    <t>10.1001/jama.2025.4486</t>
+  </si>
+  <si>
+    <t>10.1016/S0140-6736(25)00770-6</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/S0140-6736(25)00770-6</t>
+  </si>
+  <si>
+    <t>E19-E27</t>
+  </si>
+  <si>
+    <t>https://www.thelancet.com/action/showPdf?pii=S0140-6736%2825%2900770-6</t>
+  </si>
+  <si>
+    <t>10.1038/s41591-025-03668-w</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1038/s41591-025-03668-w</t>
+  </si>
+  <si>
+    <t>1784-1792</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41591-025-03668-w.pdf</t>
+  </si>
+  <si>
+    <t>10.1371/journal.pmed.1004589</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1371/journal.pmed.1004589</t>
+  </si>
+  <si>
+    <t>e1004589</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hróbjartsson A, Boutron I, Hopewell S, Moher D, Schulz F, **Collins  GS**, Tunn R, Aggarwal R, Berlin JA, Bhandari N, Butcher NJ, Campbell MK, Chidebe R, Elbourne D, Farmer A, Fergusson D, Golub RM, Goodman SN, Hoffmann T, Ioannidis JP, Kahan B, Knowles R, Lamb SE, Lewis S, Loder E, Offringa M, Ravaud P, Richards D, Rockhold FW, Schriger DL, Siegfried N, Staniszewska S, Taylor R, Thabane L, Torgerson D, Vohra S, White IR, Chan AW. </t>
+  </si>
+  <si>
+    <t>SPIRIT 2025 Explanation and Elaboration: updated guideline for protocols of randomised trials.</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1136/bmj-2024-081660</t>
+  </si>
+  <si>
+    <t>10.1136/bmj-2024-081660</t>
+  </si>
+  <si>
+    <t>e081660</t>
+  </si>
+  <si>
+    <t>https://www.bmj.com/content/389/bmj-2024-081660.full.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Safiri S, Grieger JA, Jolfayi AG, Mousavi SE, Nejadghaderi SA, Fazlollahi A, Sullman MJM, Karamzad N, Sahin F, Singh K, *Collins  GS**, Kolahi AA. </t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1186/s12937-025-01082-z</t>
+  </si>
+  <si>
+    <t>Nutrition Journal</t>
+  </si>
+  <si>
+    <t>Burden of diseases attributable to excess body weight in 204 countries and territories, 1990-2019</t>
+  </si>
+  <si>
+    <t>10.1186/s12937-025-01082-z</t>
+  </si>
+  <si>
+    <t>https://link.springer.com/content/pdf/10.1186/s12937-025-01082-z.pdf</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1471,6 +1718,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1491,41 +1761,46 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1829,7 +2104,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X63"/>
+  <dimension ref="A1:X75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.1640625" style="1" customWidth="1"/>
@@ -3073,7 +3348,7 @@
       <c r="E32" s="10" t="s">
         <v>249</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32" s="12" t="s">
         <v>250</v>
       </c>
       <c r="G32" s="1" t="s">
@@ -3088,7 +3363,7 @@
       <c r="K32" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="L32" t="s">
+      <c r="L32" s="12" t="s">
         <v>253</v>
       </c>
       <c r="X32" s="4" t="s">
@@ -3126,7 +3401,7 @@
       <c r="K33" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="L33" t="s">
+      <c r="L33" s="12" t="s">
         <v>260</v>
       </c>
       <c r="X33" s="4" t="s">
@@ -3149,7 +3424,7 @@
       <c r="E34" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="F34" s="11" t="s">
+      <c r="F34" s="13" t="s">
         <v>265</v>
       </c>
       <c r="G34" s="1" t="s">
@@ -3164,7 +3439,7 @@
       <c r="K34" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="L34" s="11" t="s">
+      <c r="L34" s="13" t="s">
         <v>271</v>
       </c>
       <c r="X34" s="4" t="s">
@@ -3187,7 +3462,7 @@
       <c r="E35" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="F35" s="11" t="s">
+      <c r="F35" s="13" t="s">
         <v>275</v>
       </c>
       <c r="G35" s="1" t="s">
@@ -3202,7 +3477,7 @@
       <c r="K35" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="L35" s="11" t="s">
+      <c r="L35" s="13" t="s">
         <v>273</v>
       </c>
       <c r="X35" s="4" t="s">
@@ -3225,7 +3500,7 @@
       <c r="E36" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="F36" s="11" t="s">
+      <c r="F36" s="13" t="s">
         <v>278</v>
       </c>
       <c r="G36" s="1" t="s">
@@ -3240,7 +3515,7 @@
       <c r="K36" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="L36" s="11" t="s">
+      <c r="L36" s="13" t="s">
         <v>282</v>
       </c>
       <c r="X36" s="4" t="s">
@@ -3263,7 +3538,7 @@
       <c r="E37" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="F37" s="11" t="s">
+      <c r="F37" s="13" t="s">
         <v>283</v>
       </c>
       <c r="G37" s="1" t="s">
@@ -3278,7 +3553,7 @@
       <c r="K37" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="L37" s="11" t="s">
+      <c r="L37" s="13" t="s">
         <v>287</v>
       </c>
       <c r="X37" s="4" t="s">
@@ -3301,7 +3576,7 @@
       <c r="E38" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="F38" s="11" t="s">
+      <c r="F38" s="13" t="s">
         <v>291</v>
       </c>
       <c r="G38" s="1" t="s">
@@ -3316,7 +3591,7 @@
       <c r="K38" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="L38" s="11" t="s">
+      <c r="L38" s="13" t="s">
         <v>290</v>
       </c>
       <c r="X38" s="4" t="s">
@@ -3339,7 +3614,7 @@
       <c r="E39" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="F39" s="11" t="s">
+      <c r="F39" s="13" t="s">
         <v>294</v>
       </c>
       <c r="G39" s="1" t="s">
@@ -3354,7 +3629,7 @@
       <c r="K39" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="L39" s="11" t="s">
+      <c r="L39" s="13" t="s">
         <v>297</v>
       </c>
       <c r="X39" s="4" t="s">
@@ -3377,7 +3652,7 @@
       <c r="E40" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="F40" s="11" t="s">
+      <c r="F40" s="13" t="s">
         <v>301</v>
       </c>
       <c r="G40" s="1" t="s">
@@ -3392,7 +3667,7 @@
       <c r="K40" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="L40" s="11" t="s">
+      <c r="L40" s="13" t="s">
         <v>305</v>
       </c>
       <c r="X40" s="4" t="s">
@@ -3415,7 +3690,7 @@
       <c r="E41" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="F41" s="11" t="s">
+      <c r="F41" s="13" t="s">
         <v>308</v>
       </c>
       <c r="G41" s="1" t="s">
@@ -3430,7 +3705,7 @@
       <c r="K41" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="L41" s="11" t="s">
+      <c r="L41" s="13" t="s">
         <v>310</v>
       </c>
       <c r="X41" s="4" t="s">
@@ -3453,7 +3728,7 @@
       <c r="E42" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="F42" s="11" t="s">
+      <c r="F42" s="13" t="s">
         <v>323</v>
       </c>
       <c r="G42" s="1" t="s">
@@ -3468,7 +3743,7 @@
       <c r="K42" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="L42" s="11" t="s">
+      <c r="L42" s="13" t="s">
         <v>314</v>
       </c>
       <c r="X42" s="4" t="s">
@@ -3491,7 +3766,7 @@
       <c r="E43" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="F43" s="11" t="s">
+      <c r="F43" s="13" t="s">
         <v>320</v>
       </c>
       <c r="G43" s="1" t="s">
@@ -3506,7 +3781,7 @@
       <c r="K43" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="L43" s="11" t="s">
+      <c r="L43" s="13" t="s">
         <v>322</v>
       </c>
       <c r="X43" s="4" t="s">
@@ -3529,7 +3804,7 @@
       <c r="E44" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="F44" s="11" t="s">
+      <c r="F44" s="13" t="s">
         <v>326</v>
       </c>
       <c r="G44" s="1" t="s">
@@ -3544,7 +3819,7 @@
       <c r="K44" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="L44" s="11" t="s">
+      <c r="L44" s="13" t="s">
         <v>329</v>
       </c>
       <c r="X44" s="4" t="s">
@@ -3567,7 +3842,7 @@
       <c r="E45" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="F45" s="11" t="s">
+      <c r="F45" s="13" t="s">
         <v>334</v>
       </c>
       <c r="G45" s="1" t="s">
@@ -3582,7 +3857,7 @@
       <c r="K45" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="L45" s="11" t="s">
+      <c r="L45" s="13" t="s">
         <v>335</v>
       </c>
       <c r="X45" s="4" t="s">
@@ -3605,7 +3880,7 @@
       <c r="E46" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="F46" s="11" t="s">
+      <c r="F46" s="13" t="s">
         <v>338</v>
       </c>
       <c r="G46" s="1" t="s">
@@ -3620,7 +3895,7 @@
       <c r="K46" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="L46" s="11" t="s">
+      <c r="L46" s="13" t="s">
         <v>342</v>
       </c>
       <c r="X46" s="4" t="s">
@@ -3643,7 +3918,7 @@
       <c r="E47" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="F47" s="11" t="s">
+      <c r="F47" s="13" t="s">
         <v>349</v>
       </c>
       <c r="G47" s="1" t="s">
@@ -3658,7 +3933,7 @@
       <c r="K47" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="L47" s="11" t="s">
+      <c r="L47" s="13" t="s">
         <v>350</v>
       </c>
       <c r="X47" s="4" t="s">
@@ -3681,7 +3956,7 @@
       <c r="E48" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="F48" s="11" t="s">
+      <c r="F48" s="13" t="s">
         <v>356</v>
       </c>
       <c r="G48" s="1" t="s">
@@ -3696,7 +3971,7 @@
       <c r="K48" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="L48" s="11" t="s">
+      <c r="L48" s="13" t="s">
         <v>358</v>
       </c>
       <c r="X48" s="4" t="s">
@@ -3719,7 +3994,7 @@
       <c r="E49" s="1" t="s">
         <v>368</v>
       </c>
-      <c r="F49" s="11" t="s">
+      <c r="F49" s="13" t="s">
         <v>369</v>
       </c>
       <c r="G49" s="1" t="s">
@@ -3737,7 +4012,7 @@
       <c r="K49" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="L49" s="11" t="s">
+      <c r="L49" s="13" t="s">
         <v>371</v>
       </c>
       <c r="X49" s="4" t="s">
@@ -3757,7 +4032,7 @@
       <c r="E50" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="F50" s="11" t="s">
+      <c r="F50" s="13" t="s">
         <v>375</v>
       </c>
       <c r="G50" s="1" t="s">
@@ -3792,7 +4067,7 @@
       <c r="E51" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="F51" s="11" t="s">
+      <c r="F51" s="13" t="s">
         <v>389</v>
       </c>
       <c r="G51" s="1" t="s">
@@ -3807,7 +4082,7 @@
       <c r="K51" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="L51" s="11" t="s">
+      <c r="L51" s="13" t="s">
         <v>381</v>
       </c>
       <c r="X51" s="4" t="s">
@@ -3830,7 +4105,7 @@
       <c r="E52" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="F52" s="11" t="s">
+      <c r="F52" s="13" t="s">
         <v>386</v>
       </c>
       <c r="G52" s="1" t="s">
@@ -3845,7 +4120,7 @@
       <c r="K52" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="L52" s="11" t="s">
+      <c r="L52" s="13" t="s">
         <v>388</v>
       </c>
       <c r="X52" s="4" t="s">
@@ -3868,7 +4143,7 @@
       <c r="E53" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="F53" s="11" t="s">
+      <c r="F53" s="13" t="s">
         <v>393</v>
       </c>
       <c r="G53" s="1" t="s">
@@ -3883,7 +4158,7 @@
       <c r="K53" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="L53" s="11" t="s">
+      <c r="L53" s="13" t="s">
         <v>396</v>
       </c>
       <c r="X53" s="4">
@@ -3906,7 +4181,7 @@
       <c r="E54" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="F54" s="11" t="s">
+      <c r="F54" s="13" t="s">
         <v>400</v>
       </c>
       <c r="G54" s="1" t="s">
@@ -3924,7 +4199,7 @@
       <c r="K54" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="L54" s="11" t="s">
+      <c r="L54" s="13" t="s">
         <v>404</v>
       </c>
       <c r="X54" s="4">
@@ -3947,7 +4222,7 @@
       <c r="E55" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="F55" s="11" t="s">
+      <c r="F55" s="13" t="s">
         <v>411</v>
       </c>
       <c r="G55" s="1" t="s">
@@ -3962,7 +4237,7 @@
       <c r="K55" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="L55" s="11" t="s">
+      <c r="L55" s="13" t="s">
         <v>409</v>
       </c>
       <c r="X55" s="4" t="s">
@@ -3985,7 +4260,7 @@
       <c r="E56" s="1" t="s">
         <v>415</v>
       </c>
-      <c r="F56" s="11" t="s">
+      <c r="F56" s="13" t="s">
         <v>418</v>
       </c>
       <c r="G56" s="1" t="s">
@@ -4000,7 +4275,7 @@
       <c r="K56" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="L56" s="11" t="s">
+      <c r="L56" s="13" t="s">
         <v>420</v>
       </c>
       <c r="X56" s="4" t="s">
@@ -4020,7 +4295,7 @@
       <c r="E57" s="1" t="s">
         <v>423</v>
       </c>
-      <c r="F57" s="11" t="s">
+      <c r="F57" s="13" t="s">
         <v>426</v>
       </c>
       <c r="G57" s="1" t="s">
@@ -4035,7 +4310,7 @@
       <c r="K57" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="L57" s="11" t="s">
+      <c r="L57" s="13" t="s">
         <v>425</v>
       </c>
       <c r="X57" s="4" t="s">
@@ -4058,7 +4333,7 @@
       <c r="E58" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="F58" s="11" t="s">
+      <c r="F58" s="13" t="s">
         <v>432</v>
       </c>
       <c r="G58" s="1" t="s">
@@ -4073,7 +4348,7 @@
       <c r="K58" s="1" t="s">
         <v>433</v>
       </c>
-      <c r="L58" s="11" t="s">
+      <c r="L58" s="13" t="s">
         <v>434</v>
       </c>
       <c r="X58" s="4">
@@ -4096,7 +4371,7 @@
       <c r="E59" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="F59" s="11" t="s">
+      <c r="F59" s="13" t="s">
         <v>438</v>
       </c>
       <c r="G59" s="1" t="s">
@@ -4111,7 +4386,7 @@
       <c r="K59" s="1" t="s">
         <v>439</v>
       </c>
-      <c r="L59" s="11" t="s">
+      <c r="L59" s="13" t="s">
         <v>440</v>
       </c>
       <c r="X59" s="4" t="s">
@@ -4131,7 +4406,7 @@
       <c r="E60" s="1" t="s">
         <v>443</v>
       </c>
-      <c r="F60" s="11" t="s">
+      <c r="F60" s="13" t="s">
         <v>445</v>
       </c>
       <c r="G60" s="1" t="s">
@@ -4166,7 +4441,7 @@
       <c r="E61" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="F61" s="11" t="s">
+      <c r="F61" s="13" t="s">
         <v>450</v>
       </c>
       <c r="G61" s="1" t="s">
@@ -4181,7 +4456,7 @@
       <c r="K61" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="L61" s="11" t="s">
+      <c r="L61" s="13" t="s">
         <v>453</v>
       </c>
       <c r="X61" s="4" t="s">
@@ -4201,7 +4476,7 @@
       <c r="E62" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="F62" s="11" t="s">
+      <c r="F62" s="13" t="s">
         <v>458</v>
       </c>
       <c r="G62" s="1" t="s">
@@ -4216,7 +4491,7 @@
       <c r="K62" s="1" t="s">
         <v>461</v>
       </c>
-      <c r="L62" s="11" t="s">
+      <c r="L62" s="13" t="s">
         <v>457</v>
       </c>
       <c r="X62" s="4" t="s">
@@ -4239,7 +4514,7 @@
       <c r="E63" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="F63" s="11" t="s">
+      <c r="F63" s="13" t="s">
         <v>467</v>
       </c>
       <c r="G63" s="1" t="s">
@@ -4254,11 +4529,464 @@
       <c r="K63" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="L63" s="11" t="s">
+      <c r="L63" s="13" t="s">
         <v>465</v>
       </c>
       <c r="X63" s="4" t="s">
         <v>469</v>
+      </c>
+    </row>
+    <row r="64" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B64" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C64" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="F64" s="13" t="s">
+        <v>472</v>
+      </c>
+      <c r="G64" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H64" s="3">
+        <v>389</v>
+      </c>
+      <c r="J64" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="K64" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="L64" s="13" t="s">
+        <v>475</v>
+      </c>
+      <c r="X64" s="4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="65" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B65" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C65" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="F65" s="13" t="s">
+        <v>477</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="H65" s="3">
+        <v>333</v>
+      </c>
+      <c r="I65" s="3">
+        <v>22</v>
+      </c>
+      <c r="J65" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="K65" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="X65" s="4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="66" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B66" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C66" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="F66" s="13" t="s">
+        <v>480</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="H66" s="3">
+        <v>31</v>
+      </c>
+      <c r="J66" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="L66" s="13" t="s">
+        <v>482</v>
+      </c>
+      <c r="X66" s="4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="67" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B67" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C67" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="F67" s="13" t="s">
+        <v>483</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="H67" s="3">
+        <v>22</v>
+      </c>
+      <c r="J67" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="K67" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="L67" s="13" t="s">
+        <v>487</v>
+      </c>
+      <c r="X67" s="4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="68" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C68" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="F68" s="13" t="s">
+        <v>490</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H68" s="3">
+        <v>389</v>
+      </c>
+      <c r="J68" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="K68" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="L68" s="13" t="s">
+        <v>489</v>
+      </c>
+      <c r="X68" s="4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="69" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B69" s="14" t="s">
+        <v>493</v>
+      </c>
+      <c r="C69" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="F69" s="13" t="s">
+        <v>497</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H69" s="3">
+        <v>389</v>
+      </c>
+      <c r="J69" s="3">
+        <v>81477</v>
+      </c>
+      <c r="K69" s="1" t="s">
+        <v>495</v>
+      </c>
+      <c r="L69" s="13" t="s">
+        <v>496</v>
+      </c>
+      <c r="X69" s="4" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="70" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B70" s="14" t="s">
+        <v>493</v>
+      </c>
+      <c r="C70" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="F70" s="13" t="s">
+        <v>499</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="H70" s="3">
+        <v>334</v>
+      </c>
+      <c r="I70" s="3">
+        <v>5</v>
+      </c>
+      <c r="J70" s="3" t="s">
+        <v>500</v>
+      </c>
+      <c r="K70" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="X70" s="4" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="71" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B71" s="14" t="s">
+        <v>493</v>
+      </c>
+      <c r="C71" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="F71" s="13" t="s">
+        <v>503</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="H71" s="3">
+        <v>405</v>
+      </c>
+      <c r="I71" s="3">
+        <v>10941</v>
+      </c>
+      <c r="J71" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="K71" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="L71" s="13" t="s">
+        <v>505</v>
+      </c>
+      <c r="X71" s="4" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="72" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B72" s="14" t="s">
+        <v>493</v>
+      </c>
+      <c r="C72" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="F72" s="13" t="s">
+        <v>507</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="H72" s="3">
+        <v>31</v>
+      </c>
+      <c r="J72" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="K72" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="L72" s="13" t="s">
+        <v>509</v>
+      </c>
+      <c r="X72" s="4" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="73" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A73" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B73" s="14" t="s">
+        <v>493</v>
+      </c>
+      <c r="C73" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="F73" s="13" t="s">
+        <v>511</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="H73" s="3">
+        <v>22</v>
+      </c>
+      <c r="J73" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="K73" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="X73" s="4" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="74" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="C74" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="F74" s="13" t="s">
+        <v>515</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H74" s="3">
+        <v>389</v>
+      </c>
+      <c r="J74" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="K74" s="14" t="s">
+        <v>516</v>
+      </c>
+      <c r="L74" s="13" t="s">
+        <v>518</v>
+      </c>
+      <c r="X74" s="4" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="75" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A75" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="C75" s="1">
+        <v>2025</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="F75" s="13" t="s">
+        <v>520</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="H75" s="3">
+        <v>24</v>
+      </c>
+      <c r="J75" s="3">
+        <v>23</v>
+      </c>
+      <c r="K75" s="1" t="s">
+        <v>523</v>
+      </c>
+      <c r="L75" s="11" t="s">
+        <v>524</v>
+      </c>
+      <c r="X75" s="4">
+        <v>2025</v>
       </c>
     </row>
   </sheetData>
@@ -4321,6 +5049,27 @@
     <hyperlink ref="F62" r:id="rId56" xr:uid="{EA92A92E-2482-3346-9BDB-B6DCB3938119}"/>
     <hyperlink ref="L63" r:id="rId57" xr:uid="{9B193542-BB08-1E4E-9C81-37218CBB33F6}"/>
     <hyperlink ref="F63" r:id="rId58" xr:uid="{637128A8-DBD2-9C45-BAEF-CC52DFED3098}"/>
+    <hyperlink ref="F64" r:id="rId59" xr:uid="{873F49F8-E75A-C748-B9FA-F188EAC80B61}"/>
+    <hyperlink ref="L64" r:id="rId60" xr:uid="{B42A90F3-4085-BA45-8055-BFADD3DEBD90}"/>
+    <hyperlink ref="F65" r:id="rId61" xr:uid="{315A43C1-28EC-C743-8468-489F2F3A0304}"/>
+    <hyperlink ref="F66" r:id="rId62" xr:uid="{C5409DF2-8262-F346-B134-D1E6FEA40E4A}"/>
+    <hyperlink ref="L66" r:id="rId63" xr:uid="{0D83BC9A-DC72-7D47-9C0F-B704DAD560B7}"/>
+    <hyperlink ref="F67" r:id="rId64" xr:uid="{59319905-C30F-0D49-9A28-E893B4F913ED}"/>
+    <hyperlink ref="L67" r:id="rId65" xr:uid="{B01D228D-6C1B-AC47-9098-AB770ED194C2}"/>
+    <hyperlink ref="L68" r:id="rId66" xr:uid="{F4082EC9-4268-6440-A03F-AB23C683BB5E}"/>
+    <hyperlink ref="F68" r:id="rId67" xr:uid="{A37B2B18-2E7A-4A4B-9C7B-F6CE8B3BBD73}"/>
+    <hyperlink ref="L69" r:id="rId68" xr:uid="{BA0D36BB-B23C-404D-8B84-4482AFA9D693}"/>
+    <hyperlink ref="F69" r:id="rId69" xr:uid="{936478F1-FB44-8C45-88BF-77CBD29D1B09}"/>
+    <hyperlink ref="F70" r:id="rId70" xr:uid="{B73D1311-0711-7A49-AFBF-7145837FE74D}"/>
+    <hyperlink ref="F71" r:id="rId71" xr:uid="{192477C9-D13E-6241-9D6C-F4B7AA577205}"/>
+    <hyperlink ref="L71" r:id="rId72" xr:uid="{6BE31E21-826B-654B-87CA-DF8AD3BC9E4F}"/>
+    <hyperlink ref="F72" r:id="rId73" xr:uid="{055938B4-AEBD-A140-9B57-2447003828AD}"/>
+    <hyperlink ref="L72" r:id="rId74" xr:uid="{1DAC8830-F129-9D4C-9F69-5B08D5A50996}"/>
+    <hyperlink ref="F73" r:id="rId75" xr:uid="{8442D49A-9211-564B-8BFE-6B058D0FA3E0}"/>
+    <hyperlink ref="F74" r:id="rId76" xr:uid="{CB417139-8722-6540-B7F6-9B6BB6C300B9}"/>
+    <hyperlink ref="L74" r:id="rId77" xr:uid="{9B88C50D-59ED-304F-BA9E-6F76D68C01BC}"/>
+    <hyperlink ref="F75" r:id="rId78" xr:uid="{439A0086-76B2-C548-88AC-9305BF14ADA1}"/>
+    <hyperlink ref="L75" r:id="rId79" xr:uid="{9029434D-DAE2-AB4C-8CB4-A4EC5FDE830B}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
updated publications from 2024 (incomplete)
</commit_message>
<xml_diff>
--- a/publications.xlsx
+++ b/publications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/g.s.collins@bham.ac.uk/git/personal_pages/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02F7D099-E7BE-964C-A2C6-8A642D6E4059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9B65542-2C2F-5344-8E74-2ED4CE153FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="46580" yWindow="600" windowWidth="22060" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="868" uniqueCount="655">
   <si>
     <t>Section</t>
   </si>
@@ -1100,9 +1100,6 @@
   </si>
   <si>
     <t>2025, reporting guideline</t>
-  </si>
-  <si>
-    <t>2025, artificial intelligence, large language models, reporting guideline</t>
   </si>
   <si>
     <t>2025, reporting guideline, CONSORT, trial</t>
@@ -1671,14 +1668,415 @@
   <si>
     <t>https://link.springer.com/content/pdf/10.1186/s12937-025-01082-z.pdf</t>
   </si>
+  <si>
+    <t>Kuo R, Freethy A, Smith J, Hill R, C J, Jerome D, Harriss E, **Collins GS**, Tutton E, Furniss D</t>
+  </si>
+  <si>
+    <t>Stakeholder perspectives towards diagnostic artificial intelligence: a co-produced qualitative evidence synthesis</t>
+  </si>
+  <si>
+    <t>2024-03-21</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.eclinm.2024.102555</t>
+  </si>
+  <si>
+    <t>10.1016/j.eclinm.2024.102555</t>
+  </si>
+  <si>
+    <t>https://www.thelancet.com/action/showPdf?pii=S2589-5370%2824%2900134-2</t>
+  </si>
+  <si>
+    <t>eClinicalMedicine</t>
+  </si>
+  <si>
+    <t>2024, artificial intelligence</t>
+  </si>
+  <si>
+    <t>Duarte RV, Bresnahan R, Copley S, Eldabe S, Thomson S, North RB, Baranidharan G, Levy RM, **Collins GS**, Taylor RS</t>
+  </si>
+  <si>
+    <t>Reporting guidelines for randomised clinical trial reports of implantable neurostimulation devices the CONSORT-iNeurostim extension</t>
+  </si>
+  <si>
+    <t>2024-11-12</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.eclinm.2024.102932</t>
+  </si>
+  <si>
+    <t>10.1016/j.eclinm.2024.102932 External Link</t>
+  </si>
+  <si>
+    <t>https://www.thelancet.com/action/showPdf?pii=S2589-5370%2824%2900511-X</t>
+  </si>
+  <si>
+    <t>2024, reporting guideline, trials, CONSORT</t>
+  </si>
+  <si>
+    <t>Bresnahan R, Copley S, Eldabe S, Thomson S, North RB, Baranidharan G, Levy RM, **Collins GS**, Taylor RS, Duarte R</t>
+  </si>
+  <si>
+    <t>10.1016/j.eclinm.2024.102933</t>
+  </si>
+  <si>
+    <t>Reporting guidelines for protocols of randomised clinical trial of implantable neurostimulation devices the SPIRIT-iNeurostim extension</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.eclinm.2024.102933</t>
+  </si>
+  <si>
+    <t>https://www.thelancet.com/action/showPdf?pii=S2589-5370%2824%2900512-1</t>
+  </si>
+  <si>
+    <t>Whittle R, Ensor J, Hattle M, Dhiman P, **Collins GS**, Riley RD</t>
+  </si>
+  <si>
+    <t>Calculating the power of planned individual participant data meta-analysis to examine a prognostic factor effect of a binary outcome</t>
+  </si>
+  <si>
+    <t>2024-07-24</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1002/jrsm.1737</t>
+  </si>
+  <si>
+    <t>Research Synthesis Methods</t>
+  </si>
+  <si>
+    <t>905-916</t>
+  </si>
+  <si>
+    <t>10.1002/jrsm.1737</t>
+  </si>
+  <si>
+    <t>https://onlinelibrary.wiley.com/doi/epdf/10.1002/jrsm.1737</t>
+  </si>
+  <si>
+    <t>2024, meta-analysis, prognostic factor</t>
+  </si>
+  <si>
+    <t>Manyara AM, Purvis A, Ciani O, **Collins GS**, Taylor RS</t>
+  </si>
+  <si>
+    <t>Sample size in multistakeholder Delphi surveys: at what minimum sample size to replicability of results stabilise</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.jclinepi.2024.111485</t>
+  </si>
+  <si>
+    <t>2024-07-22</t>
+  </si>
+  <si>
+    <t>10.1016/j.jclinepi.2024.111485</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/pii/S0895435624002415/pdfft?md5=642e28f48c9dfe7c9dbae414acc18fe8&amp;pid=1-s2.0-S0895435624002415-main.pdf</t>
+  </si>
+  <si>
+    <t>2024, delphi surveys, sample size</t>
+  </si>
+  <si>
+    <t>The CHART collaborative [includes **Collins GS**]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protocol for the development of the Chatbot Assessment Reporting Tool (CHART) for clinical advice. </t>
+  </si>
+  <si>
+    <t>2024-05-21</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1136/bmjopen-2023-081155</t>
+  </si>
+  <si>
+    <t>10.1136/bmjopen-2023-081155</t>
+  </si>
+  <si>
+    <t>e081155</t>
+  </si>
+  <si>
+    <t>https://bmjopen.bmj.com/content/bmjopen/14/5/e081155.full.pdf</t>
+  </si>
+  <si>
+    <t>2024, artificial intelligence, CHART, large language models, protocol</t>
+  </si>
+  <si>
+    <t>2025, artificial intelligence, large language models, reporting guideline, CHART</t>
+  </si>
+  <si>
+    <t>Riley RD, **Collins GS**, Kirton L, Snell K, Ensor J, Whittle R, Dhiman P, van Smeden M, Liu X, Nirantharakumar K, Manson-Whitton J, Westwood AJ, Cazier JP, Moons KGM, Martin G, Sperrin M, Denniston A, Harrell Jr FE, Archer L.</t>
+  </si>
+  <si>
+    <t>Uncertainty of individual risk from clinical prediction models: rationale, challenges, and approaches</t>
+  </si>
+  <si>
+    <t>2025-02-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.1136/bmj-2024-080749 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1136/bmj-2024-080749 </t>
+  </si>
+  <si>
+    <t>e080749</t>
+  </si>
+  <si>
+    <t>https://www.bmj.com/content/388/bmj-2024-080749.full.pdf</t>
+  </si>
+  <si>
+    <t>2025, prediction models, uncertainty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andaur Navarro CL, Damen JAA, Ghannad M, Dhiman P, van Smeden M, Reitsma JB, **Collins  GS**, Riley RD, Moons KGM, Hooft L. </t>
+  </si>
+  <si>
+    <t>2024-05-14</t>
+  </si>
+  <si>
+    <t>SPIN-PM: a consensus framework to evaluate the spin in studies on prediction models</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.jclinepi.2024.111364</t>
+  </si>
+  <si>
+    <t>10.1016/j.jclinepi.2024.111364</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/pii/S0895435624001197/pdfft?md5=6344e1b49dfeff35290e18ac90314fc2&amp;pid=1-s2.0-S0895435624001197-main.pdf</t>
+  </si>
+  <si>
+    <t>2024, prediction models, spin</t>
+  </si>
+  <si>
+    <t>Moher D, **Collins GS**, Hoffmann T, Glasziou P, Ravaud P, Bian ZX</t>
+  </si>
+  <si>
+    <t>2024-08-13</t>
+  </si>
+  <si>
+    <t>Reporting on data sharing: executive position of the EQUATOR Network</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1136/bmj-2024-079694</t>
+  </si>
+  <si>
+    <t>e079694</t>
+  </si>
+  <si>
+    <t>10.1136/bmj-2024-079694</t>
+  </si>
+  <si>
+    <t>https://www.bmj.com/content/386/bmj-2024-079694.full.pdf</t>
+  </si>
+  <si>
+    <t>2024, EQUATOR, data sharing</t>
+  </si>
+  <si>
+    <t>White N, Parsons R, Borg D, **Collins GS**, Barnett A</t>
+  </si>
+  <si>
+    <t>Planned but ever published? A retrospective analysis of clinical prediction modelling studies posted on clinicaltrials.gov between 2000 and 2020</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/pii/S0895435624001884/pdfft?md5=d0f55c36c4813563a70de1d8ad0c993a&amp;pid=1-s2.0-S0895435624001884-main.pdf</t>
+  </si>
+  <si>
+    <t>2024-07-09</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.jclinepi.2024.111433</t>
+  </si>
+  <si>
+    <t>10.1016/j.jclinepi.2024.111433</t>
+  </si>
+  <si>
+    <t>2024, prediction models, meta-research</t>
+  </si>
+  <si>
+    <t>Safiri S, Hassanzadeh K, Jolfayi AG, Mousavi SE, Asghari KM, Nejadghaderi SA, Naghdi-Sedeh N, Noori M, Sullman MJM, **Collins GS**, Kolahi AA</t>
+  </si>
+  <si>
+    <t>Kidney cancer in the Middle East and North Africa region: a 30-year analysis (1990-2019).</t>
+  </si>
+  <si>
+    <t>2024-06-10</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1038/s41598-024-64521-7</t>
+  </si>
+  <si>
+    <t>10.1038/s41598-024-64521-7</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41598-024-64521-7.pdf</t>
+  </si>
+  <si>
+    <t>Scientific Reports</t>
+  </si>
+  <si>
+    <t>Logullo P, de Beyer JA, Kirtley S, Schlüssel MM, **Collins  GS**</t>
+  </si>
+  <si>
+    <t>Open access journal publication in open health science: benefits, challenges, and limitations</t>
+  </si>
+  <si>
+    <t>2024-07-23</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1136/bmjebm-2022-112126</t>
+  </si>
+  <si>
+    <t>BMJ Evidence-Mased Medicine</t>
+  </si>
+  <si>
+    <t>223-228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1136/bmjebm-2022-112126
+</t>
+  </si>
+  <si>
+    <t>https://ebm.bmj.com/content/ebmed/29/4/223.full.pdf?with-ds=yes</t>
+  </si>
+  <si>
+    <t>2024, open access</t>
+  </si>
+  <si>
+    <t>Self A, Schlüssel M, **Collins  GS**, Dhombres F, Fries N, Haddad G, Salomon LJ, Massoud M, Papageorghiou AT</t>
+  </si>
+  <si>
+    <t>External validation of models to estimate gestational age in the second and third trimester using ultrasound: a prospective multicentre observational study</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1111/1471-0528.17922</t>
+  </si>
+  <si>
+    <t>2024-08-08</t>
+  </si>
+  <si>
+    <t>BJOG</t>
+  </si>
+  <si>
+    <t>1862-1873</t>
+  </si>
+  <si>
+    <t>10.1111/1471-0528.17922</t>
+  </si>
+  <si>
+    <t>https://obgyn.onlinelibrary.wiley.com/doi/epdf/10.1111/1471-0528.17922</t>
+  </si>
+  <si>
+    <t>2024, prediction models, validation</t>
+  </si>
+  <si>
+    <t>Riley RD, Ensor J, Snell K, Archer L, Whittle R, Dhiman P, Alderman J, Liu X, Nirantharakumar K, Kirton L, van Smeden M, Moons KG, Cazier JB, Denniston AK, Van Calster B, **Collins GS**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The importance of sample size on the quality and utility of prediction models for healthcare. </t>
+  </si>
+  <si>
+    <t>2024-06-02</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.landig.2025.01.013</t>
+  </si>
+  <si>
+    <t>10.1016/j.landig.2025.01.013 </t>
+  </si>
+  <si>
+    <t>https://www.thelancet.com/action/showPdf?pii=S2589-7500%2825%2900021-4</t>
+  </si>
+  <si>
+    <t>2024, prediction models, sample size</t>
+  </si>
+  <si>
+    <t>Safiri S, Noori M, Nejadghaderi SA, Shamekh, Sullman MJM, **Collins GS**, Kolahi AA</t>
+  </si>
+  <si>
+    <t>The burden of schizophrenia in the Middle East and North Africa region, 1990-2019</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41598-024-59905-8.pdf</t>
+  </si>
+  <si>
+    <t>10.1038/s41598-024-59905-8</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1038/s41598-024-59905-8</t>
+  </si>
+  <si>
+    <t>2024-04-27</t>
+  </si>
+  <si>
+    <t>Østengaard L, Barrientos A, Boutron I, Chan AW, **Collins  GS**, Franco M, Hopewell S, Moher D, Muthurajah A, Nejstgaard CH, Schulz KF, Speich B, Tang E, Tunn R, Watanabe N, Xu C, Hróbjartsson A</t>
+  </si>
+  <si>
+    <t>Development of a topic-specific bibliographic database supporting the updates of SPIRIT 2013 and CONSORT 2010</t>
+  </si>
+  <si>
+    <t>2024-05-15</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1002/cesm.12057</t>
+  </si>
+  <si>
+    <t>Cochrane Evidence Synthesis and Methods</t>
+  </si>
+  <si>
+    <t>e12057</t>
+  </si>
+  <si>
+    <t>10.1002/cesm.12057</t>
+  </si>
+  <si>
+    <t>https://onlinelibrary.wiley.com/doi/epdf/10.1002/cesm.12057</t>
+  </si>
+  <si>
+    <t>2024, trials, CONSORT, SPIRIT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reinke A, Tizabi MD, Baumgartner M, Eisenmann M, Heckmann-Notzel D, Kavu E, Radsh T, Sudre CH, Acion L, Antonelli M, Arbel T, Bakas S, Benis A, Blascko M, Buttner F, Cardoso MJ, Cheplyguba V, Chen J, Christodolou E, Cimini BA, **Collins GS**, Farahani K, Ferrer L, Galdran A, van Ginneken B, Blocker B, Godau P, Haase R, Hashimoto DA, Hoffman MM, Huisman M, Isensee F, Jannin P, Kahn CE, Kainmueller D, Kainz B, Karagyris A, Karthikesalingam A, Kenngott H, Kleesiek J, Kofler F, Kooi T, Kopp-Schneider A, Kozubek M, Kreshuk A, Kurc T, Landman BA, Litjens G, Madani A, Maier-Hein L, Martel AL, Mattson P, Meijering E, Menze B, Moons KGM, Muller H, Nichyporuk B, Nickel F, Petersen J, Rafelski SM, Rajpoot N, Reyes M, Riegler MA, Rieke N, Saez-Rodriguez J, Sanchez CI, Shetty S, van Smeden M, Summers RM, Taha AA, Tiulpin A, Tsaftaris SA, Van Calster B, Varoquaux G, Wiesenfarth M, Yaniv ZR, Jager PF, Maier-Hein L. </t>
+  </si>
+  <si>
+    <t>Metrics reloaded: recommendations for image analysis validation</t>
+  </si>
+  <si>
+    <t>2024-02-12</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1038/s41592-023-02151-z</t>
+  </si>
+  <si>
+    <t>10.1038/s41592-023-02151-z</t>
+  </si>
+  <si>
+    <t>Nature Methods</t>
+  </si>
+  <si>
+    <t>195-212</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41592-023-02151-z.pdf</t>
+  </si>
+  <si>
+    <t>2024, validation, image analysis</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1761,46 +2159,50 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2104,7 +2506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X75"/>
+  <dimension ref="A1:X92"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.1640625" style="1" customWidth="1"/>
@@ -2236,7 +2638,7 @@
         <v>40</v>
       </c>
       <c r="X2" s="4" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="3" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2277,7 +2679,7 @@
         <v>50</v>
       </c>
       <c r="X3" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="4" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2312,7 +2714,7 @@
         <v>34</v>
       </c>
       <c r="X4" s="4" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="5" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2657,7 +3059,7 @@
         <v>113</v>
       </c>
       <c r="X13" s="4" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="14" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2762,7 +3164,7 @@
         <v>134</v>
       </c>
       <c r="X16" s="4" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="17" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3250,7 +3652,7 @@
         <v>231</v>
       </c>
       <c r="X29" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="30" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3288,7 +3690,7 @@
         <v>241</v>
       </c>
       <c r="X30" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="31" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3443,7 +3845,7 @@
         <v>271</v>
       </c>
       <c r="X34" s="4" t="s">
-        <v>360</v>
+        <v>568</v>
       </c>
     </row>
     <row r="35" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3481,7 +3883,7 @@
         <v>273</v>
       </c>
       <c r="X35" s="4" t="s">
-        <v>360</v>
+        <v>568</v>
       </c>
     </row>
     <row r="36" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3519,7 +3921,7 @@
         <v>282</v>
       </c>
       <c r="X36" s="4" t="s">
-        <v>360</v>
+        <v>568</v>
       </c>
     </row>
     <row r="37" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3557,7 +3959,7 @@
         <v>287</v>
       </c>
       <c r="X37" s="4" t="s">
-        <v>360</v>
+        <v>568</v>
       </c>
     </row>
     <row r="38" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3595,7 +3997,7 @@
         <v>290</v>
       </c>
       <c r="X38" s="4" t="s">
-        <v>360</v>
+        <v>568</v>
       </c>
     </row>
     <row r="39" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3633,7 +4035,7 @@
         <v>297</v>
       </c>
       <c r="X39" s="4" t="s">
-        <v>360</v>
+        <v>568</v>
       </c>
     </row>
     <row r="40" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3671,7 +4073,7 @@
         <v>305</v>
       </c>
       <c r="X40" s="4" t="s">
-        <v>360</v>
+        <v>568</v>
       </c>
     </row>
     <row r="41" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3709,7 +4111,7 @@
         <v>310</v>
       </c>
       <c r="X41" s="4" t="s">
-        <v>360</v>
+        <v>568</v>
       </c>
     </row>
     <row r="42" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3747,7 +4149,7 @@
         <v>314</v>
       </c>
       <c r="X42" s="4" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="43" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3823,7 +4225,7 @@
         <v>329</v>
       </c>
       <c r="X44" s="4" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="45" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -3983,19 +4385,19 @@
         <v>27</v>
       </c>
       <c r="B49" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="C49" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D49" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="C49" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D49" s="2" t="s">
+      <c r="E49" s="1" t="s">
         <v>367</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="F49" s="13" t="s">
         <v>368</v>
-      </c>
-      <c r="F49" s="13" t="s">
-        <v>369</v>
       </c>
       <c r="G49" s="1" t="s">
         <v>97</v>
@@ -4010,13 +4412,13 @@
         <v>100873</v>
       </c>
       <c r="K49" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="L49" s="13" t="s">
         <v>370</v>
       </c>
-      <c r="L49" s="13" t="s">
+      <c r="X49" s="4" t="s">
         <v>371</v>
-      </c>
-      <c r="X49" s="4" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="50" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4024,28 +4426,28 @@
         <v>27</v>
       </c>
       <c r="B50" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="C50" s="1">
+        <v>2025</v>
+      </c>
+      <c r="E50" s="1" t="s">
         <v>373</v>
       </c>
-      <c r="C50" s="1">
-        <v>2025</v>
-      </c>
-      <c r="E50" s="1" t="s">
+      <c r="F50" s="13" t="s">
         <v>374</v>
       </c>
-      <c r="F50" s="13" t="s">
+      <c r="G50" s="1" t="s">
         <v>375</v>
-      </c>
-      <c r="G50" s="1" t="s">
-        <v>376</v>
       </c>
       <c r="H50" s="3">
         <v>93</v>
       </c>
       <c r="J50" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="K50" s="1" t="s">
         <v>377</v>
-      </c>
-      <c r="K50" s="1" t="s">
-        <v>378</v>
       </c>
       <c r="X50" s="4">
         <v>2025</v>
@@ -4056,7 +4458,7 @@
         <v>27</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C51" s="1">
         <v>2025</v>
@@ -4065,10 +4467,10 @@
         <v>204</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F51" s="13" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="G51" s="1" t="s">
         <v>207</v>
@@ -4080,10 +4482,10 @@
         <v>167</v>
       </c>
       <c r="K51" s="1" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="L51" s="13" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="X51" s="4" t="s">
         <v>90</v>
@@ -4094,7 +4496,7 @@
         <v>27</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C52" s="1">
         <v>2025</v>
@@ -4103,10 +4505,10 @@
         <v>161</v>
       </c>
       <c r="E52" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="F52" s="13" t="s">
         <v>385</v>
-      </c>
-      <c r="F52" s="13" t="s">
-        <v>386</v>
       </c>
       <c r="G52" s="1" t="s">
         <v>33</v>
@@ -4118,10 +4520,10 @@
         <v>111833</v>
       </c>
       <c r="K52" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="L52" s="13" t="s">
         <v>387</v>
-      </c>
-      <c r="L52" s="13" t="s">
-        <v>388</v>
       </c>
       <c r="X52" s="4" t="s">
         <v>90</v>
@@ -4132,22 +4534,22 @@
         <v>27</v>
       </c>
       <c r="B53" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="C53" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="E53" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="C53" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D53" s="2" t="s">
+      <c r="F53" s="13" t="s">
         <v>392</v>
       </c>
-      <c r="E53" s="1" t="s">
-        <v>391</v>
-      </c>
-      <c r="F53" s="13" t="s">
+      <c r="G53" s="1" t="s">
         <v>393</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>394</v>
       </c>
       <c r="H53" s="3">
         <v>116</v>
@@ -4156,10 +4558,10 @@
         <v>105749</v>
       </c>
       <c r="K53" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="L53" s="13" t="s">
         <v>395</v>
-      </c>
-      <c r="L53" s="13" t="s">
-        <v>396</v>
       </c>
       <c r="X53" s="4">
         <v>2025</v>
@@ -4170,22 +4572,22 @@
         <v>27</v>
       </c>
       <c r="B54" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="C54" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D54" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="C54" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D54" s="2" t="s">
+      <c r="E54" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="E54" s="1" t="s">
+      <c r="F54" s="13" t="s">
         <v>399</v>
       </c>
-      <c r="F54" s="13" t="s">
+      <c r="G54" s="1" t="s">
         <v>400</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>401</v>
       </c>
       <c r="H54" s="3">
         <v>192</v>
@@ -4194,13 +4596,13 @@
         <v>5</v>
       </c>
       <c r="J54" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="K54" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="K54" s="1" t="s">
+      <c r="L54" s="13" t="s">
         <v>403</v>
-      </c>
-      <c r="L54" s="13" t="s">
-        <v>404</v>
       </c>
       <c r="X54" s="4">
         <v>2025</v>
@@ -4211,19 +4613,19 @@
         <v>27</v>
       </c>
       <c r="B55" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="C55" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="E55" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="C55" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D55" s="2" t="s">
+      <c r="F55" s="13" t="s">
         <v>410</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>408</v>
-      </c>
-      <c r="F55" s="13" t="s">
-        <v>411</v>
       </c>
       <c r="G55" s="1" t="s">
         <v>207</v>
@@ -4235,13 +4637,13 @@
         <v>71</v>
       </c>
       <c r="K55" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="L55" s="13" t="s">
+        <v>408</v>
+      </c>
+      <c r="X55" s="4" t="s">
         <v>412</v>
-      </c>
-      <c r="L55" s="13" t="s">
-        <v>409</v>
-      </c>
-      <c r="X55" s="4" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="56" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4249,19 +4651,19 @@
         <v>27</v>
       </c>
       <c r="B56" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="C56" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="E56" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="C56" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>419</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>415</v>
-      </c>
       <c r="F56" s="13" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="G56" s="1" t="s">
         <v>38</v>
@@ -4270,16 +4672,16 @@
         <v>388</v>
       </c>
       <c r="J56" s="3" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="K56" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="L56" s="13" t="s">
+        <v>419</v>
+      </c>
+      <c r="X56" s="4" t="s">
         <v>420</v>
-      </c>
-      <c r="X56" s="4" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="57" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4287,31 +4689,31 @@
         <v>27</v>
       </c>
       <c r="B57" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="C57" s="1">
+        <v>2025</v>
+      </c>
+      <c r="E57" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="C57" s="1">
-        <v>2025</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>423</v>
-      </c>
       <c r="F57" s="13" t="s">
+        <v>425</v>
+      </c>
+      <c r="G57" s="1" t="s">
         <v>426</v>
-      </c>
-      <c r="G57" s="1" t="s">
-        <v>427</v>
       </c>
       <c r="H57" s="3">
         <v>57</v>
       </c>
       <c r="J57" s="3" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="K57" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="L57" s="13" t="s">
         <v>424</v>
-      </c>
-      <c r="L57" s="13" t="s">
-        <v>425</v>
       </c>
       <c r="X57" s="4" t="s">
         <v>359</v>
@@ -4322,19 +4724,19 @@
         <v>27</v>
       </c>
       <c r="B58" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="C58" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E58" s="1" t="s">
         <v>429</v>
       </c>
-      <c r="C58" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D58" s="2" t="s">
+      <c r="F58" s="13" t="s">
         <v>431</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="F58" s="13" t="s">
-        <v>432</v>
       </c>
       <c r="G58" s="1" t="s">
         <v>288</v>
@@ -4346,10 +4748,10 @@
         <v>180</v>
       </c>
       <c r="K58" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="L58" s="13" t="s">
         <v>433</v>
-      </c>
-      <c r="L58" s="13" t="s">
-        <v>434</v>
       </c>
       <c r="X58" s="4">
         <v>2025</v>
@@ -4360,19 +4762,19 @@
         <v>27</v>
       </c>
       <c r="B59" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="C59" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="E59" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="C59" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D59" s="2" t="s">
+      <c r="F59" s="13" t="s">
         <v>437</v>
-      </c>
-      <c r="E59" s="1" t="s">
-        <v>436</v>
-      </c>
-      <c r="F59" s="13" t="s">
-        <v>438</v>
       </c>
       <c r="G59" s="1" t="s">
         <v>38</v>
@@ -4384,13 +4786,13 @@
         <v>81554</v>
       </c>
       <c r="K59" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="L59" s="13" t="s">
         <v>439</v>
       </c>
-      <c r="L59" s="13" t="s">
+      <c r="X59" s="4" t="s">
         <v>440</v>
-      </c>
-      <c r="X59" s="4" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="60" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4398,28 +4800,28 @@
         <v>27</v>
       </c>
       <c r="B60" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="C60" s="1">
+        <v>2025</v>
+      </c>
+      <c r="E60" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="C60" s="1">
-        <v>2025</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>443</v>
-      </c>
       <c r="F60" s="13" t="s">
+        <v>444</v>
+      </c>
+      <c r="G60" s="1" t="s">
         <v>445</v>
-      </c>
-      <c r="G60" s="1" t="s">
-        <v>446</v>
       </c>
       <c r="H60" s="3">
         <v>36</v>
       </c>
       <c r="J60" s="3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="K60" s="1" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="X60" s="4">
         <v>2025</v>
@@ -4436,13 +4838,13 @@
         <v>2025</v>
       </c>
       <c r="D61" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="F61" s="13" t="s">
         <v>449</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>448</v>
-      </c>
-      <c r="F61" s="13" t="s">
-        <v>450</v>
       </c>
       <c r="G61" s="1" t="s">
         <v>339</v>
@@ -4451,16 +4853,16 @@
         <v>31</v>
       </c>
       <c r="J61" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="K61" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="K61" s="1" t="s">
+      <c r="L61" s="13" t="s">
         <v>452</v>
       </c>
-      <c r="L61" s="13" t="s">
+      <c r="X61" s="4" t="s">
         <v>453</v>
-      </c>
-      <c r="X61" s="4" t="s">
-        <v>454</v>
       </c>
     </row>
     <row r="62" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4468,34 +4870,34 @@
         <v>27</v>
       </c>
       <c r="B62" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="C62" s="1">
+        <v>2025</v>
+      </c>
+      <c r="E62" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="C62" s="1">
-        <v>2025</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>456</v>
-      </c>
       <c r="F62" s="13" t="s">
+        <v>457</v>
+      </c>
+      <c r="G62" s="1" t="s">
         <v>458</v>
-      </c>
-      <c r="G62" s="1" t="s">
-        <v>459</v>
       </c>
       <c r="H62" s="3">
         <v>121</v>
       </c>
       <c r="J62" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="K62" s="1" t="s">
         <v>460</v>
       </c>
-      <c r="K62" s="1" t="s">
+      <c r="L62" s="13" t="s">
+        <v>456</v>
+      </c>
+      <c r="X62" s="4" t="s">
         <v>461</v>
-      </c>
-      <c r="L62" s="13" t="s">
-        <v>457</v>
-      </c>
-      <c r="X62" s="4" t="s">
-        <v>462</v>
       </c>
     </row>
     <row r="63" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4503,19 +4905,19 @@
         <v>27</v>
       </c>
       <c r="B63" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="C63" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="E63" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="C63" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D63" s="2" t="s">
+      <c r="F63" s="13" t="s">
         <v>466</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>464</v>
-      </c>
-      <c r="F63" s="13" t="s">
-        <v>467</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>33</v>
@@ -4527,13 +4929,13 @@
         <v>111675</v>
       </c>
       <c r="K63" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="L63" s="13" t="s">
+        <v>464</v>
+      </c>
+      <c r="X63" s="4" t="s">
         <v>468</v>
-      </c>
-      <c r="L63" s="13" t="s">
-        <v>465</v>
-      </c>
-      <c r="X63" s="4" t="s">
-        <v>469</v>
       </c>
     </row>
     <row r="64" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4547,13 +4949,13 @@
         <v>2025</v>
       </c>
       <c r="D64" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="E64" s="1" t="s">
         <v>470</v>
       </c>
-      <c r="E64" s="1" t="s">
+      <c r="F64" s="13" t="s">
         <v>471</v>
-      </c>
-      <c r="F64" s="13" t="s">
-        <v>472</v>
       </c>
       <c r="G64" s="1" t="s">
         <v>38</v>
@@ -4562,16 +4964,16 @@
         <v>389</v>
       </c>
       <c r="J64" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="K64" s="1" t="s">
         <v>473</v>
       </c>
-      <c r="K64" s="1" t="s">
+      <c r="L64" s="13" t="s">
         <v>474</v>
       </c>
-      <c r="L64" s="13" t="s">
-        <v>475</v>
-      </c>
       <c r="X64" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="65" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4585,13 +4987,13 @@
         <v>2025</v>
       </c>
       <c r="D65" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="E65" s="1" t="s">
         <v>470</v>
       </c>
-      <c r="E65" s="1" t="s">
-        <v>471</v>
-      </c>
       <c r="F65" s="13" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="G65" s="1" t="s">
         <v>128</v>
@@ -4603,13 +5005,13 @@
         <v>22</v>
       </c>
       <c r="J65" s="3" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="K65" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="X65" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="66" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4623,13 +5025,13 @@
         <v>2025</v>
       </c>
       <c r="D66" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="E66" s="1" t="s">
         <v>470</v>
       </c>
-      <c r="E66" s="1" t="s">
-        <v>471</v>
-      </c>
       <c r="F66" s="13" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="G66" s="1" t="s">
         <v>339</v>
@@ -4638,16 +5040,16 @@
         <v>31</v>
       </c>
       <c r="J66" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="L66" s="13" t="s">
         <v>481</v>
       </c>
-      <c r="K66" s="1" t="s">
-        <v>479</v>
-      </c>
-      <c r="L66" s="13" t="s">
-        <v>482</v>
-      </c>
       <c r="X66" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="67" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4661,31 +5063,31 @@
         <v>2025</v>
       </c>
       <c r="D67" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="E67" s="1" t="s">
         <v>470</v>
       </c>
-      <c r="E67" s="1" t="s">
-        <v>471</v>
-      </c>
       <c r="F67" s="13" t="s">
+        <v>482</v>
+      </c>
+      <c r="G67" s="1" t="s">
         <v>483</v>
-      </c>
-      <c r="G67" s="1" t="s">
-        <v>484</v>
       </c>
       <c r="H67" s="3">
         <v>22</v>
       </c>
       <c r="J67" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="K67" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="K67" s="1" t="s">
+      <c r="L67" s="13" t="s">
         <v>486</v>
       </c>
-      <c r="L67" s="13" t="s">
-        <v>487</v>
-      </c>
       <c r="X67" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="68" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4699,13 +5101,13 @@
         <v>2025</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="F68" s="13" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="G68" s="1" t="s">
         <v>38</v>
@@ -4714,16 +5116,16 @@
         <v>389</v>
       </c>
       <c r="J68" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="K68" s="1" t="s">
         <v>491</v>
       </c>
-      <c r="K68" s="1" t="s">
-        <v>492</v>
-      </c>
       <c r="L68" s="13" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="X68" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="69" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4731,19 +5133,19 @@
         <v>27</v>
       </c>
       <c r="B69" s="14" t="s">
+        <v>492</v>
+      </c>
+      <c r="C69" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="E69" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="C69" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D69" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="E69" s="1" t="s">
-        <v>494</v>
-      </c>
       <c r="F69" s="13" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>38</v>
@@ -4755,13 +5157,13 @@
         <v>81477</v>
       </c>
       <c r="K69" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="L69" s="13" t="s">
         <v>495</v>
       </c>
-      <c r="L69" s="13" t="s">
-        <v>496</v>
-      </c>
       <c r="X69" s="4" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="70" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4769,19 +5171,19 @@
         <v>27</v>
       </c>
       <c r="B70" s="14" t="s">
+        <v>492</v>
+      </c>
+      <c r="C70" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="E70" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="C70" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="E70" s="1" t="s">
-        <v>494</v>
-      </c>
       <c r="F70" s="13" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="G70" s="1" t="s">
         <v>128</v>
@@ -4793,13 +5195,13 @@
         <v>5</v>
       </c>
       <c r="J70" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="K70" s="1" t="s">
         <v>500</v>
       </c>
-      <c r="K70" s="1" t="s">
-        <v>501</v>
-      </c>
       <c r="X70" s="4" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="71" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4807,19 +5209,19 @@
         <v>27</v>
       </c>
       <c r="B71" s="14" t="s">
+        <v>492</v>
+      </c>
+      <c r="C71" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="E71" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="C71" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="E71" s="1" t="s">
-        <v>494</v>
-      </c>
       <c r="F71" s="13" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="G71" s="1" t="s">
         <v>47</v>
@@ -4831,16 +5233,16 @@
         <v>10941</v>
       </c>
       <c r="J71" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="K71" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="L71" s="13" t="s">
         <v>504</v>
       </c>
-      <c r="K71" s="1" t="s">
-        <v>502</v>
-      </c>
-      <c r="L71" s="13" t="s">
-        <v>505</v>
-      </c>
       <c r="X71" s="4" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="72" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4848,19 +5250,19 @@
         <v>27</v>
       </c>
       <c r="B72" s="14" t="s">
+        <v>492</v>
+      </c>
+      <c r="C72" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="E72" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="C72" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="E72" s="1" t="s">
-        <v>494</v>
-      </c>
       <c r="F72" s="13" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="G72" s="1" t="s">
         <v>339</v>
@@ -4869,16 +5271,16 @@
         <v>31</v>
       </c>
       <c r="J72" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="K72" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="L72" s="13" t="s">
         <v>508</v>
       </c>
-      <c r="K72" s="1" t="s">
-        <v>506</v>
-      </c>
-      <c r="L72" s="13" t="s">
-        <v>509</v>
-      </c>
       <c r="X72" s="4" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="73" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4886,34 +5288,34 @@
         <v>27</v>
       </c>
       <c r="B73" s="14" t="s">
+        <v>492</v>
+      </c>
+      <c r="C73" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="E73" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="C73" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="E73" s="1" t="s">
-        <v>494</v>
-      </c>
       <c r="F73" s="13" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="H73" s="3">
         <v>22</v>
       </c>
       <c r="J73" s="3" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="K73" s="1" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="X73" s="4" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="74" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4921,19 +5323,19 @@
         <v>27</v>
       </c>
       <c r="B74" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="C74" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="E74" s="1" t="s">
         <v>513</v>
       </c>
-      <c r="C74" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="E74" s="1" t="s">
+      <c r="F74" s="13" t="s">
         <v>514</v>
-      </c>
-      <c r="F74" s="13" t="s">
-        <v>515</v>
       </c>
       <c r="G74" s="1" t="s">
         <v>38</v>
@@ -4942,16 +5344,16 @@
         <v>389</v>
       </c>
       <c r="J74" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="K74" s="14" t="s">
+        <v>515</v>
+      </c>
+      <c r="L74" s="13" t="s">
         <v>517</v>
       </c>
-      <c r="K74" s="14" t="s">
-        <v>516</v>
-      </c>
-      <c r="L74" s="13" t="s">
-        <v>518</v>
-      </c>
       <c r="X74" s="4" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="75" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -4959,19 +5361,19 @@
         <v>27</v>
       </c>
       <c r="B75" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="C75" s="1">
+        <v>2025</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="F75" s="13" t="s">
         <v>519</v>
       </c>
-      <c r="C75" s="1">
-        <v>2025</v>
-      </c>
-      <c r="E75" s="1" t="s">
-        <v>522</v>
-      </c>
-      <c r="F75" s="13" t="s">
+      <c r="G75" s="1" t="s">
         <v>520</v>
-      </c>
-      <c r="G75" s="1" t="s">
-        <v>521</v>
       </c>
       <c r="H75" s="3">
         <v>24</v>
@@ -4980,13 +5382,662 @@
         <v>23</v>
       </c>
       <c r="K75" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="L75" s="11" t="s">
         <v>523</v>
       </c>
-      <c r="L75" s="11" t="s">
+      <c r="X75" s="4">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="76" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A76" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B76" s="1" t="s">
         <v>524</v>
       </c>
-      <c r="X75" s="4">
-        <v>2025</v>
+      <c r="C76" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>525</v>
+      </c>
+      <c r="F76" s="11" t="s">
+        <v>527</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="H76" s="3">
+        <v>71</v>
+      </c>
+      <c r="J76" s="3">
+        <v>102555</v>
+      </c>
+      <c r="K76" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="L76" s="11" t="s">
+        <v>529</v>
+      </c>
+      <c r="X76" s="4" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="77" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A77" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="C77" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="F77" s="11" t="s">
+        <v>535</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="H77" s="3">
+        <v>78</v>
+      </c>
+      <c r="J77" s="3">
+        <v>102932</v>
+      </c>
+      <c r="K77" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="L77" s="11" t="s">
+        <v>537</v>
+      </c>
+      <c r="X77" s="4" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="78" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="C78" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="F78" s="11" t="s">
+        <v>542</v>
+      </c>
+      <c r="G78" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="H78" s="3">
+        <v>78</v>
+      </c>
+      <c r="J78" s="3">
+        <v>102933</v>
+      </c>
+      <c r="K78" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="L78" s="11" t="s">
+        <v>543</v>
+      </c>
+      <c r="X78" s="4" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="79" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A79" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="C79" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="H79" s="3">
+        <v>15</v>
+      </c>
+      <c r="J79" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="K79" s="1" t="s">
+        <v>550</v>
+      </c>
+      <c r="L79" s="11" t="s">
+        <v>551</v>
+      </c>
+      <c r="X79" s="4" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="80" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A80" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C80" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>556</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="F80" s="11" t="s">
+        <v>555</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H80" s="3">
+        <v>174</v>
+      </c>
+      <c r="J80" s="3">
+        <v>111485</v>
+      </c>
+      <c r="K80" s="1" t="s">
+        <v>557</v>
+      </c>
+      <c r="L80" s="11" t="s">
+        <v>558</v>
+      </c>
+      <c r="X80" s="4" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="81" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="C81" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>561</v>
+      </c>
+      <c r="F81" s="11" t="s">
+        <v>563</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H81" s="3">
+        <v>14</v>
+      </c>
+      <c r="J81" s="3" t="s">
+        <v>565</v>
+      </c>
+      <c r="K81" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="L81" s="11" t="s">
+        <v>566</v>
+      </c>
+      <c r="X81" s="4" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="82" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A82" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>569</v>
+      </c>
+      <c r="C82" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>570</v>
+      </c>
+      <c r="F82" s="11" t="s">
+        <v>572</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H82" s="3">
+        <v>388</v>
+      </c>
+      <c r="J82" s="3" t="s">
+        <v>574</v>
+      </c>
+      <c r="K82" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="L82" s="11" t="s">
+        <v>575</v>
+      </c>
+      <c r="X82" s="4" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="83" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>577</v>
+      </c>
+      <c r="C83" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>579</v>
+      </c>
+      <c r="F83" s="11" t="s">
+        <v>580</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H83" s="3">
+        <v>170</v>
+      </c>
+      <c r="J83" s="3">
+        <v>111364</v>
+      </c>
+      <c r="K83" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="L83" s="11" t="s">
+        <v>582</v>
+      </c>
+      <c r="X83" s="4" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="84" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A84" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>584</v>
+      </c>
+      <c r="C84" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>586</v>
+      </c>
+      <c r="F84" s="11" t="s">
+        <v>587</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H84" s="3">
+        <v>386</v>
+      </c>
+      <c r="J84" s="3" t="s">
+        <v>588</v>
+      </c>
+      <c r="K84" s="1" t="s">
+        <v>589</v>
+      </c>
+      <c r="L84" s="11" t="s">
+        <v>590</v>
+      </c>
+      <c r="X84" s="4" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="85" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A85" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>592</v>
+      </c>
+      <c r="C85" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>593</v>
+      </c>
+      <c r="F85" s="11" t="s">
+        <v>596</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H85" s="3">
+        <v>173</v>
+      </c>
+      <c r="J85" s="3">
+        <v>111433</v>
+      </c>
+      <c r="K85" s="1" t="s">
+        <v>597</v>
+      </c>
+      <c r="L85" s="11" t="s">
+        <v>594</v>
+      </c>
+      <c r="X85" s="4" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="86" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A86" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>599</v>
+      </c>
+      <c r="C86" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="E86" s="1" t="s">
+        <v>600</v>
+      </c>
+      <c r="F86" s="11" t="s">
+        <v>602</v>
+      </c>
+      <c r="G86" s="1" t="s">
+        <v>605</v>
+      </c>
+      <c r="H86" s="3">
+        <v>14</v>
+      </c>
+      <c r="J86" s="3">
+        <v>13710</v>
+      </c>
+      <c r="K86" s="1" t="s">
+        <v>603</v>
+      </c>
+      <c r="L86" s="11" t="s">
+        <v>604</v>
+      </c>
+      <c r="X86" s="4">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="87" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A87" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>606</v>
+      </c>
+      <c r="C87" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>608</v>
+      </c>
+      <c r="E87" s="1" t="s">
+        <v>607</v>
+      </c>
+      <c r="F87" s="11" t="s">
+        <v>609</v>
+      </c>
+      <c r="G87" s="1" t="s">
+        <v>610</v>
+      </c>
+      <c r="H87" s="3">
+        <v>29</v>
+      </c>
+      <c r="J87" s="3" t="s">
+        <v>611</v>
+      </c>
+      <c r="K87" s="16" t="s">
+        <v>612</v>
+      </c>
+      <c r="L87" s="11" t="s">
+        <v>613</v>
+      </c>
+      <c r="X87" s="4" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="88" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A88" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>615</v>
+      </c>
+      <c r="C88" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="E88" s="1" t="s">
+        <v>616</v>
+      </c>
+      <c r="F88" s="11" t="s">
+        <v>617</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>619</v>
+      </c>
+      <c r="H88" s="3">
+        <v>131</v>
+      </c>
+      <c r="J88" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="K88" s="1" t="s">
+        <v>621</v>
+      </c>
+      <c r="L88" s="11" t="s">
+        <v>622</v>
+      </c>
+      <c r="X88" s="4" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="89" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A89" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>624</v>
+      </c>
+      <c r="C89" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="E89" s="1" t="s">
+        <v>625</v>
+      </c>
+      <c r="F89" s="11" t="s">
+        <v>627</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="H89" s="3">
+        <v>7</v>
+      </c>
+      <c r="I89" s="3">
+        <v>6</v>
+      </c>
+      <c r="J89" s="3">
+        <v>100857</v>
+      </c>
+      <c r="K89" s="15" t="s">
+        <v>628</v>
+      </c>
+      <c r="L89" s="11" t="s">
+        <v>629</v>
+      </c>
+      <c r="X89" s="4" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="90" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A90" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>631</v>
+      </c>
+      <c r="C90" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>632</v>
+      </c>
+      <c r="F90" s="11" t="s">
+        <v>635</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>605</v>
+      </c>
+      <c r="H90" s="3">
+        <v>14</v>
+      </c>
+      <c r="J90" s="3">
+        <v>9720</v>
+      </c>
+      <c r="K90" s="1" t="s">
+        <v>634</v>
+      </c>
+      <c r="L90" s="11" t="s">
+        <v>633</v>
+      </c>
+      <c r="X90" s="4">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="91" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A91" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>637</v>
+      </c>
+      <c r="C91" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>638</v>
+      </c>
+      <c r="F91" s="11" t="s">
+        <v>640</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>641</v>
+      </c>
+      <c r="H91" s="3">
+        <v>2</v>
+      </c>
+      <c r="J91" s="3" t="s">
+        <v>642</v>
+      </c>
+      <c r="K91" s="1" t="s">
+        <v>643</v>
+      </c>
+      <c r="L91" s="11" t="s">
+        <v>644</v>
+      </c>
+      <c r="X91" s="4" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="92" spans="1:24" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A92" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>646</v>
+      </c>
+      <c r="C92" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>648</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>647</v>
+      </c>
+      <c r="F92" s="11" t="s">
+        <v>649</v>
+      </c>
+      <c r="G92" s="1" t="s">
+        <v>651</v>
+      </c>
+      <c r="H92" s="3">
+        <v>21</v>
+      </c>
+      <c r="J92" s="3" t="s">
+        <v>652</v>
+      </c>
+      <c r="K92" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="L92" s="11" t="s">
+        <v>653</v>
+      </c>
+      <c r="X92" s="4" t="s">
+        <v>654</v>
       </c>
     </row>
   </sheetData>
@@ -5070,6 +6121,40 @@
     <hyperlink ref="L74" r:id="rId77" xr:uid="{9B88C50D-59ED-304F-BA9E-6F76D68C01BC}"/>
     <hyperlink ref="F75" r:id="rId78" xr:uid="{439A0086-76B2-C548-88AC-9305BF14ADA1}"/>
     <hyperlink ref="L75" r:id="rId79" xr:uid="{9029434D-DAE2-AB4C-8CB4-A4EC5FDE830B}"/>
+    <hyperlink ref="F76" r:id="rId80" xr:uid="{F199D265-EA0C-FB4E-BCC7-021DB0ED0244}"/>
+    <hyperlink ref="L76" r:id="rId81" xr:uid="{4F00E1C2-6FB0-AB41-A668-9950D4D7413D}"/>
+    <hyperlink ref="F77" r:id="rId82" xr:uid="{7FC35840-31AA-9548-8ACF-B4598324B8A5}"/>
+    <hyperlink ref="L77" r:id="rId83" xr:uid="{3A01E82C-68EC-1947-8AE1-CA9E4D072CFC}"/>
+    <hyperlink ref="F78" r:id="rId84" xr:uid="{1AD2F1BF-7DE0-7D44-A5E5-71643AC424A9}"/>
+    <hyperlink ref="L78" r:id="rId85" xr:uid="{46AA21EA-D77B-CC42-9676-0FE637DDFD8A}"/>
+    <hyperlink ref="L79" r:id="rId86" xr:uid="{34ACB49B-5DF3-E748-88F0-6B300A52781D}"/>
+    <hyperlink ref="F80" r:id="rId87" xr:uid="{B8C773D8-75C5-E84D-85A8-82D4DA37E5FB}"/>
+    <hyperlink ref="L80" r:id="rId88" xr:uid="{C291A886-816E-384F-B7D7-E35ADE84925A}"/>
+    <hyperlink ref="F81" r:id="rId89" xr:uid="{226A6538-537D-2941-80A2-B4BFEDFFCD00}"/>
+    <hyperlink ref="L81" r:id="rId90" xr:uid="{A1427B85-4965-5D45-9EE9-32D3A25B6500}"/>
+    <hyperlink ref="F82" r:id="rId91" xr:uid="{81107602-D18D-0F46-B8D5-A5C951B6525E}"/>
+    <hyperlink ref="L82" r:id="rId92" xr:uid="{E7AF7748-8115-144C-BB5C-54B3EAF901CA}"/>
+    <hyperlink ref="F83" r:id="rId93" xr:uid="{2E4E292D-4FD0-EB43-B557-9F7B3EF63536}"/>
+    <hyperlink ref="L83" r:id="rId94" xr:uid="{3E06EE77-1D5A-404C-99B7-7383B6A27BD8}"/>
+    <hyperlink ref="F84" r:id="rId95" xr:uid="{595ED802-041A-C949-AC8F-26774353CF85}"/>
+    <hyperlink ref="L84" r:id="rId96" xr:uid="{026C1530-AD69-9C4C-8900-31DBFABD113E}"/>
+    <hyperlink ref="L85" r:id="rId97" xr:uid="{915DFA38-2E3E-9F47-B369-62B0012069AC}"/>
+    <hyperlink ref="F85" r:id="rId98" xr:uid="{41CF7726-FF72-3F4F-BE5F-334142A96C9B}"/>
+    <hyperlink ref="F86" r:id="rId99" xr:uid="{A23F774A-5C09-0148-A2AD-F4D9407C38FF}"/>
+    <hyperlink ref="L86" r:id="rId100" xr:uid="{B80EC81C-8FBD-9047-969D-888EB967E0FF}"/>
+    <hyperlink ref="F87" r:id="rId101" xr:uid="{8388F7FD-267D-3C40-907A-3BCE3E6FCF8C}"/>
+    <hyperlink ref="L87" r:id="rId102" xr:uid="{CCC4F84F-CA4E-EB41-9486-C74C58FA2A77}"/>
+    <hyperlink ref="F88" r:id="rId103" xr:uid="{6DAD25BE-FAD6-8646-9AEF-7127DA05A22F}"/>
+    <hyperlink ref="L88" r:id="rId104" xr:uid="{50962D4E-5C18-AF48-B48C-F3D39A71AB2F}"/>
+    <hyperlink ref="F89" r:id="rId105" xr:uid="{2184B4A6-92CC-1F4E-BD74-78F529EAFCE0}"/>
+    <hyperlink ref="K89" r:id="rId106" display="https://doi.org/10.1016/j.landig.2025.01.013" xr:uid="{295AD83C-640C-FF4A-B83D-1AA914C59427}"/>
+    <hyperlink ref="L89" r:id="rId107" xr:uid="{05E4EB16-6549-3146-90A5-118AD64457E4}"/>
+    <hyperlink ref="L90" r:id="rId108" xr:uid="{7EB059B3-541B-D547-9054-DEA7FA720582}"/>
+    <hyperlink ref="F90" r:id="rId109" xr:uid="{41D07154-CB5C-7849-AF1A-03DDA67595B7}"/>
+    <hyperlink ref="F91" r:id="rId110" xr:uid="{3479FDB3-B82F-6E40-95F2-C0AE935CABF8}"/>
+    <hyperlink ref="L91" r:id="rId111" xr:uid="{BDF3EB00-6548-524D-B2EF-A8466C4DCBFD}"/>
+    <hyperlink ref="F92" r:id="rId112" xr:uid="{9A50E123-633E-6C41-BD84-2843ED62376E}"/>
+    <hyperlink ref="L92" r:id="rId113" xr:uid="{6D9DDF97-4D91-4546-9DF7-79DC65F89AC1}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>